<commit_message>
feat: expose parent entity columns in child table views and fix upward join logic
- Updated ENTITY_COLUMN_TREE so every child entity table can display columns from its full ancestor chain up to Robot (e.g. batteries table can now show plastic, communication, and robot columns)
- Fixed TableViewService._buildJoinClauses to support upward joins when a non-root entity is the base table; the previous implementation assumed robots was always the root and generated invalid SQL when traversing child→parent relationships
- Updated parser port to 8999 in start.bat

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/files/files/battery_upload_1_report.xlsx
+++ b/app/files/files/battery_upload_1_report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>robot_UUID</t>
   </si>
@@ -38,9 +38,6 @@
   </si>
   <si>
     <t>lithium_version</t>
-  </si>
-  <si>
-    <t>notes</t>
   </si>
   <si>
     <t>robot-bat-001</t>
@@ -472,13 +469,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="10" width="22" customWidth="1"/>
+    <col min="1" max="9" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -506,72 +503,63 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>9</v>
       </c>
+      <c r="B2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" t="s">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" t="s">
         <v>13</v>
       </c>
-      <c r="E2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" t="s">
-        <v>17</v>
-      </c>
-      <c r="I2" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2">
-        <v>12345</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>22</v>
       </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>24</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>25</v>
-      </c>
-      <c r="I3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3">
-        <v>1234555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>